<commit_message>
win rate 52.7 profit factor 0.99
</commit_message>
<xml_diff>
--- a/EddiewareOpeningRangeSetup/EddiewareOpeningRangeSetup/Score_indicator_results_from_root_folder.xlsx
+++ b/EddiewareOpeningRangeSetup/EddiewareOpeningRangeSetup/Score_indicator_results_from_root_folder.xlsx
@@ -2,24 +2,24 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
-  <workbookProtection/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="1560" yWindow="1560" windowWidth="18900" windowHeight="10965" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
-  <calcPr calcId="124519" fullCalcOnLoad="1"/>
+  <calcPr calcId="191029" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="1">
-    <numFmt numFmtId="164" formatCode="+0.##;-0.##;0"/>
+  <numFmts count="2">
+    <numFmt numFmtId="164" formatCode="\+0.##;\-0.##;0"/>
+    <numFmt numFmtId="165" formatCode="+0.##;-0.##;0"/>
   </numFmts>
-  <fonts count="2">
+  <fonts count="4">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -28,15 +28,33 @@
       <scheme val="minor"/>
     </font>
     <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <color theme="1"/>
+      <sz val="11"/>
+      <u val="single"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
       <b val="1"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFD9EAF7"/>
+      </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
@@ -56,15 +74,18 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="10" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
@@ -427,23 +448,23 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AJ13"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <dimension ref="A1:AJ26"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15"/>
   <cols>
-    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="1" max="3"/>
     <col width="12" customWidth="1" min="2" max="2"/>
     <col width="12" customWidth="1" min="3" max="3"/>
     <col width="10" customWidth="1" min="4" max="4"/>
     <col width="14" customWidth="1" min="5" max="5"/>
     <col width="10" customWidth="1" min="6" max="6"/>
-    <col width="14" customWidth="1" min="7" max="7"/>
+    <col width="14" customWidth="1" min="7" max="8"/>
     <col width="14" customWidth="1" min="8" max="8"/>
-    <col width="12" customWidth="1" min="9" max="9"/>
+    <col width="12" customWidth="1" min="9" max="12"/>
     <col width="12" customWidth="1" min="10" max="10"/>
     <col width="12" customWidth="1" min="11" max="11"/>
     <col width="12" customWidth="1" min="12" max="12"/>
     <col width="16" customWidth="1" min="13" max="13"/>
-    <col width="10" customWidth="1" min="14" max="14"/>
+    <col width="10" customWidth="1" min="14" max="17"/>
     <col width="10" customWidth="1" min="15" max="15"/>
     <col width="10" customWidth="1" min="16" max="16"/>
     <col width="10" customWidth="1" min="17" max="17"/>
@@ -463,191 +484,191 @@
     </row>
     <row r="2">
       <c r="A2" s="1">
-        <f>IF((COUNTIF(Q4:Q13,"&gt;0")+COUNTIF(Q4:Q13,"&lt;0"))=0,"",COUNTIF(Q4:Q13,"&gt;0")/(COUNTIF(Q4:Q13,"&gt;0")+COUNTIF(Q4:Q13,"&lt;0")))</f>
+        <f>IF((COUNTIF(Q4:Q26,"&gt;0")+COUNTIF(Q4:Q26,"&lt;0"))=0,"",COUNTIF(Q4:Q26,"&gt;0")/(COUNTIF(Q4:Q26,"&gt;0")+COUNTIF(Q4:Q26,"&lt;0")))</f>
         <v/>
       </c>
       <c r="B2" s="2">
-        <f>IF(ABS(SUMIF(Q4:Q13,"&lt;0",Q4:Q13))=0,IF(SUMIF(Q4:Q13,"&gt;0",Q4:Q13)&gt;0,"INF",""),SUMIF(Q4:Q13,"&gt;0",Q4:Q13)/ABS(SUMIF(Q4:Q13,"&lt;0",Q4:Q13)))</f>
+        <f>IF(ABS(SUMIF(Q4:Q26,"&lt;0",Q4:Q26))=0,IF(SUMIF(Q4:Q26,"&gt;0",Q4:Q26)&gt;0,"INF",""),SUMIF(Q4:Q26,"&gt;0",Q4:Q26)/ABS(SUMIF(Q4:Q26,"&lt;0",Q4:Q26)))</f>
         <v/>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="3" t="inlineStr">
+      <c r="A3" s="6" t="inlineStr">
         <is>
           <t>fecha</t>
         </is>
       </c>
-      <c r="B3" s="3" t="inlineStr">
+      <c r="B3" s="6" t="inlineStr">
         <is>
           <t>or_low</t>
         </is>
       </c>
-      <c r="C3" s="3" t="inlineStr">
+      <c r="C3" s="6" t="inlineStr">
         <is>
           <t>or_high</t>
         </is>
       </c>
-      <c r="D3" s="3" t="inlineStr">
+      <c r="D3" s="6" t="inlineStr">
         <is>
           <t>range</t>
         </is>
       </c>
-      <c r="E3" s="3" t="inlineStr">
+      <c r="E3" s="6" t="inlineStr">
         <is>
           <t>VWAP_entry</t>
         </is>
       </c>
-      <c r="F3" s="3" t="inlineStr">
+      <c r="F3" s="6" t="inlineStr">
         <is>
           <t>Body</t>
         </is>
       </c>
-      <c r="G3" s="3" t="inlineStr">
+      <c r="G3" s="6" t="inlineStr">
         <is>
           <t>Volume_entry</t>
         </is>
       </c>
-      <c r="H3" s="3" t="inlineStr">
+      <c r="H3" s="6" t="inlineStr">
         <is>
           <t>Delta_entry</t>
         </is>
       </c>
-      <c r="I3" s="3" t="inlineStr">
+      <c r="I3" s="6" t="inlineStr">
         <is>
           <t>BreakOut_SPEED</t>
         </is>
       </c>
-      <c r="J3" s="3" t="inlineStr">
+      <c r="J3" s="6" t="inlineStr">
         <is>
           <t>BreakOut_TICKS_PER_SEC</t>
         </is>
       </c>
-      <c r="K3" s="3" t="inlineStr">
+      <c r="K3" s="6" t="inlineStr">
         <is>
           <t>score total</t>
         </is>
       </c>
-      <c r="L3" s="3" t="inlineStr">
+      <c r="L3" s="6" t="inlineStr">
         <is>
           <t>SL_price</t>
         </is>
       </c>
-      <c r="M3" s="3" t="inlineStr">
+      <c r="M3" s="6" t="inlineStr">
         <is>
           <t>Entry_price</t>
         </is>
       </c>
-      <c r="N3" s="3" t="inlineStr">
+      <c r="N3" s="6" t="inlineStr">
         <is>
           <t>TP_price</t>
         </is>
       </c>
-      <c r="O3" s="3" t="inlineStr">
+      <c r="O3" s="6" t="inlineStr">
         <is>
           <t>SL_ticks</t>
         </is>
       </c>
-      <c r="P3" s="3" t="inlineStr">
+      <c r="P3" s="6" t="inlineStr">
         <is>
           <t>TP_ticks</t>
         </is>
       </c>
-      <c r="Q3" s="3" t="inlineStr">
+      <c r="Q3" s="6" t="inlineStr">
         <is>
           <t>result TP SL BE</t>
         </is>
       </c>
-      <c r="R3" s="3" t="inlineStr">
+      <c r="R3" s="6" t="inlineStr">
         <is>
           <t>Side</t>
         </is>
       </c>
-      <c r="S3" s="3" t="inlineStr">
+      <c r="S3" s="6" t="inlineStr">
         <is>
           <t>Speed_Profile</t>
         </is>
       </c>
-      <c r="T3" s="3" t="inlineStr">
+      <c r="T3" s="6" t="inlineStr">
         <is>
           <t>MAE_ticks</t>
         </is>
       </c>
-      <c r="U3" s="3" t="inlineStr">
+      <c r="U3" s="6" t="inlineStr">
         <is>
           <t>MFE_ticks</t>
         </is>
       </c>
-      <c r="V3" s="3" t="inlineStr">
+      <c r="V3" s="6" t="inlineStr">
         <is>
           <t>Exporter_VERSION</t>
         </is>
       </c>
-      <c r="W3" s="3" t="inlineStr">
+      <c r="W3" s="6" t="inlineStr">
         <is>
           <t>EntryTime_NY</t>
         </is>
       </c>
-      <c r="X3" s="3" t="inlineStr">
+      <c r="X3" s="6" t="inlineStr">
         <is>
           <t>EntryBar</t>
         </is>
       </c>
-      <c r="Y3" s="3" t="inlineStr">
+      <c r="Y3" s="6" t="inlineStr">
         <is>
           <t>Speed_Elapsed_SECONDS</t>
         </is>
       </c>
-      <c r="Z3" s="3" t="inlineStr">
+      <c r="Z3" s="6" t="inlineStr">
         <is>
           <t>Speed_Replay_Fallback</t>
         </is>
       </c>
-      <c r="AA3" s="3" t="inlineStr">
+      <c r="AA3" s="6" t="inlineStr">
         <is>
           <t>Speed_Timing_Source</t>
         </is>
       </c>
-      <c r="AB3" s="3" t="inlineStr">
+      <c r="AB3" s="6" t="inlineStr">
         <is>
           <t>Range_OK</t>
         </is>
       </c>
-      <c r="AC3" s="3" t="inlineStr">
+      <c r="AC3" s="6" t="inlineStr">
         <is>
           <t>Body_OK</t>
         </is>
       </c>
-      <c r="AD3" s="3" t="inlineStr">
+      <c r="AD3" s="6" t="inlineStr">
         <is>
           <t>Volume_OK</t>
         </is>
       </c>
-      <c r="AE3" s="3" t="inlineStr">
+      <c r="AE3" s="6" t="inlineStr">
         <is>
           <t>Delta_OK</t>
         </is>
       </c>
-      <c r="AF3" s="3" t="inlineStr">
+      <c r="AF3" s="6" t="inlineStr">
         <is>
           <t>Time_OK</t>
         </is>
       </c>
-      <c r="AG3" s="3" t="inlineStr">
+      <c r="AG3" s="6" t="inlineStr">
         <is>
           <t>VWAP_OK</t>
         </is>
       </c>
-      <c r="AH3" s="3" t="inlineStr">
+      <c r="AH3" s="6" t="inlineStr">
         <is>
           <t>Speed_OK</t>
         </is>
       </c>
-      <c r="AI3" s="3" t="inlineStr">
+      <c r="AI3" s="6" t="inlineStr">
         <is>
           <t>Result_Label</t>
         </is>
       </c>
-      <c r="AJ3" s="3" t="inlineStr">
+      <c r="AJ3" s="6" t="inlineStr">
         <is>
           <t>Exit_price</t>
         </is>
@@ -656,74 +677,74 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2026-05-11</t>
+          <t>2026-04-21</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>29282.5</v>
+        <v>26772.5</v>
       </c>
       <c r="C4" t="n">
-        <v>29346.25</v>
+        <v>26827.5</v>
       </c>
       <c r="D4" t="n">
-        <v>255</v>
+        <v>220</v>
       </c>
       <c r="E4" t="n">
-        <v>29316.26</v>
+        <v>26835.25</v>
       </c>
       <c r="F4" t="n">
-        <v>5</v>
+        <v>55</v>
       </c>
       <c r="G4" t="n">
-        <v>103</v>
+        <v>1713</v>
       </c>
       <c r="H4" t="n">
-        <v>25</v>
+        <v>-435</v>
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>A+ speed</t>
+          <t>normal speed</t>
         </is>
       </c>
       <c r="J4" t="n">
-        <v>12.52</v>
+        <v>2.25</v>
       </c>
       <c r="K4" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="L4" t="n">
-        <v>29322.5</v>
+        <v>26773.75</v>
       </c>
       <c r="M4" t="n">
-        <v>29347.5</v>
+        <v>26758.75</v>
       </c>
       <c r="N4" t="n">
-        <v>29377.5</v>
+        <v>26728.75</v>
       </c>
       <c r="O4" t="n">
-        <v>100</v>
+        <v>60</v>
       </c>
       <c r="P4" t="n">
         <v>120</v>
       </c>
-      <c r="Q4" s="4" t="n">
-        <v>120</v>
+      <c r="Q4" s="7" t="n">
+        <v>20</v>
       </c>
       <c r="R4" t="inlineStr">
         <is>
-          <t>BUY</t>
+          <t>SELL</t>
         </is>
       </c>
       <c r="S4" t="inlineStr">
         <is>
-          <t>BUY</t>
+          <t>SELL1</t>
         </is>
       </c>
       <c r="T4" t="n">
-        <v>5</v>
+        <v>30</v>
       </c>
       <c r="U4" t="n">
-        <v>120</v>
+        <v>40</v>
       </c>
       <c r="V4" t="inlineStr">
         <is>
@@ -736,10 +757,10 @@
         </is>
       </c>
       <c r="X4" t="n">
-        <v>2311</v>
+        <v>2310</v>
       </c>
       <c r="Y4" t="n">
-        <v>0.3994</v>
+        <v>24.4818</v>
       </c>
       <c r="Z4" t="inlineStr">
         <is>
@@ -758,12 +779,12 @@
       </c>
       <c r="AC4" t="inlineStr">
         <is>
-          <t>FALSE</t>
+          <t>TRUE</t>
         </is>
       </c>
       <c r="AD4" t="inlineStr">
         <is>
-          <t>FALSE</t>
+          <t>TRUE</t>
         </is>
       </c>
       <c r="AE4" t="inlineStr">
@@ -788,84 +809,84 @@
       </c>
       <c r="AI4" t="inlineStr">
         <is>
-          <t>TP</t>
+          <t>EXIT</t>
         </is>
       </c>
       <c r="AJ4" t="n">
-        <v>29377.5</v>
+        <v>26753.75</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-05-12</t>
+          <t>2026-04-22</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>29146.25</v>
+        <v>26852.5</v>
       </c>
       <c r="C5" t="n">
-        <v>29227.5</v>
+        <v>26893.75</v>
       </c>
       <c r="D5" t="n">
-        <v>325</v>
+        <v>165</v>
       </c>
       <c r="E5" t="n">
-        <v>29202.57</v>
+        <v>26841.85</v>
       </c>
       <c r="F5" t="n">
-        <v>10</v>
+        <v>70</v>
       </c>
       <c r="G5" t="n">
-        <v>44</v>
+        <v>1300</v>
       </c>
       <c r="H5" t="n">
-        <v>-4</v>
+        <v>-120</v>
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>A+ speed</t>
+          <t>normal speed</t>
         </is>
       </c>
       <c r="J5" t="n">
-        <v>23.77</v>
+        <v>2.1</v>
       </c>
       <c r="K5" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="L5" t="n">
-        <v>29205</v>
+        <v>26836.25</v>
       </c>
       <c r="M5" t="n">
-        <v>29230</v>
+        <v>26821.25</v>
       </c>
       <c r="N5" t="n">
-        <v>29260</v>
+        <v>26791.25</v>
       </c>
       <c r="O5" t="n">
-        <v>100</v>
+        <v>60</v>
       </c>
       <c r="P5" t="n">
         <v>120</v>
       </c>
-      <c r="Q5" s="4" t="n">
-        <v>120</v>
+      <c r="Q5" s="7" t="n">
+        <v>-60</v>
       </c>
       <c r="R5" t="inlineStr">
         <is>
-          <t>BUY</t>
+          <t>SELL</t>
         </is>
       </c>
       <c r="S5" t="inlineStr">
         <is>
-          <t>BUY</t>
+          <t>SELL1</t>
         </is>
       </c>
       <c r="T5" t="n">
         <v>65</v>
       </c>
       <c r="U5" t="n">
-        <v>120</v>
+        <v>30</v>
       </c>
       <c r="V5" t="inlineStr">
         <is>
@@ -874,14 +895,14 @@
       </c>
       <c r="W5" t="inlineStr">
         <is>
-          <t>09:40:00</t>
+          <t>09:33:00</t>
         </is>
       </c>
       <c r="X5" t="n">
-        <v>2320</v>
+        <v>2312</v>
       </c>
       <c r="Y5" t="n">
-        <v>0.4207</v>
+        <v>33.2933</v>
       </c>
       <c r="Z5" t="inlineStr">
         <is>
@@ -905,12 +926,12 @@
       </c>
       <c r="AD5" t="inlineStr">
         <is>
-          <t>FALSE</t>
+          <t>TRUE</t>
         </is>
       </c>
       <c r="AE5" t="inlineStr">
         <is>
-          <t>FALSE</t>
+          <t>TRUE</t>
         </is>
       </c>
       <c r="AF5" t="inlineStr">
@@ -930,39 +951,39 @@
       </c>
       <c r="AI5" t="inlineStr">
         <is>
-          <t>TP</t>
+          <t>SL</t>
         </is>
       </c>
       <c r="AJ5" t="n">
-        <v>29260</v>
+        <v>26836.25</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2026-05-13</t>
+          <t>2026-04-23</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>29252.5</v>
+        <v>26965</v>
       </c>
       <c r="C6" t="n">
-        <v>29288.75</v>
+        <v>27016.25</v>
       </c>
       <c r="D6" t="n">
-        <v>145</v>
+        <v>205</v>
       </c>
       <c r="E6" t="n">
-        <v>29321.36</v>
+        <v>26995.97</v>
       </c>
       <c r="F6" t="n">
-        <v>35</v>
+        <v>40</v>
       </c>
       <c r="G6" t="n">
-        <v>1114</v>
+        <v>802</v>
       </c>
       <c r="H6" t="n">
-        <v>-176</v>
+        <v>162</v>
       </c>
       <c r="I6" t="inlineStr">
         <is>
@@ -970,19 +991,19 @@
         </is>
       </c>
       <c r="J6" t="n">
-        <v>2.08</v>
+        <v>2.32</v>
       </c>
       <c r="K6" t="n">
         <v>7</v>
       </c>
       <c r="L6" t="n">
-        <v>29258.75</v>
+        <v>27051.25</v>
       </c>
       <c r="M6" t="n">
-        <v>29243.75</v>
+        <v>27066.25</v>
       </c>
       <c r="N6" t="n">
-        <v>29213.75</v>
+        <v>27096.25</v>
       </c>
       <c r="O6" t="n">
         <v>60</v>
@@ -990,24 +1011,24 @@
       <c r="P6" t="n">
         <v>120</v>
       </c>
-      <c r="Q6" s="4" t="n">
-        <v>30</v>
+      <c r="Q6" s="7" t="n">
+        <v>25</v>
       </c>
       <c r="R6" t="inlineStr">
         <is>
-          <t>SELL</t>
+          <t>BUY</t>
         </is>
       </c>
       <c r="S6" t="inlineStr">
         <is>
-          <t>SELL1</t>
+          <t>BUY1</t>
         </is>
       </c>
       <c r="T6" t="n">
-        <v>0</v>
+        <v>20</v>
       </c>
       <c r="U6" t="n">
-        <v>60</v>
+        <v>50</v>
       </c>
       <c r="V6" t="inlineStr">
         <is>
@@ -1016,14 +1037,14 @@
       </c>
       <c r="W6" t="inlineStr">
         <is>
-          <t>09:31:00</t>
+          <t>09:46:00</t>
         </is>
       </c>
       <c r="X6" t="n">
-        <v>2311</v>
+        <v>2326</v>
       </c>
       <c r="Y6" t="n">
-        <v>16.8169</v>
+        <v>17.2107</v>
       </c>
       <c r="Z6" t="inlineStr">
         <is>
@@ -1076,64 +1097,64 @@
         </is>
       </c>
       <c r="AJ6" t="n">
-        <v>29236.25</v>
+        <v>27072.5</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2026-05-14</t>
+          <t>2026-04-24</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>29460</v>
+        <v>27176.25</v>
       </c>
       <c r="C7" t="n">
-        <v>29492.5</v>
+        <v>27223.75</v>
       </c>
       <c r="D7" t="n">
-        <v>130</v>
+        <v>190</v>
       </c>
       <c r="E7" t="n">
-        <v>29543.51</v>
+        <v>27208.66</v>
       </c>
       <c r="F7" t="n">
-        <v>65</v>
+        <v>75</v>
       </c>
       <c r="G7" t="n">
-        <v>801</v>
+        <v>1287</v>
       </c>
       <c r="H7" t="n">
-        <v>263</v>
+        <v>173</v>
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>A+ speed</t>
+          <t>normal speed</t>
         </is>
       </c>
       <c r="J7" t="n">
-        <v>11.01</v>
+        <v>2.06</v>
       </c>
       <c r="K7" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="L7" t="n">
-        <v>29490</v>
+        <v>27228.75</v>
       </c>
       <c r="M7" t="n">
-        <v>29515</v>
+        <v>27243.75</v>
       </c>
       <c r="N7" t="n">
-        <v>29545</v>
+        <v>27273.75</v>
       </c>
       <c r="O7" t="n">
-        <v>100</v>
+        <v>60</v>
       </c>
       <c r="P7" t="n">
         <v>120</v>
       </c>
-      <c r="Q7" s="4" t="n">
-        <v>120</v>
+      <c r="Q7" s="7" t="n">
+        <v>-60</v>
       </c>
       <c r="R7" t="inlineStr">
         <is>
@@ -1142,14 +1163,14 @@
       </c>
       <c r="S7" t="inlineStr">
         <is>
-          <t>BUY</t>
+          <t>BUY1</t>
         </is>
       </c>
       <c r="T7" t="n">
-        <v>25</v>
+        <v>60</v>
       </c>
       <c r="U7" t="n">
-        <v>120</v>
+        <v>10</v>
       </c>
       <c r="V7" t="inlineStr">
         <is>
@@ -1158,14 +1179,14 @@
       </c>
       <c r="W7" t="inlineStr">
         <is>
-          <t>09:32:00</t>
+          <t>09:34:00</t>
         </is>
       </c>
       <c r="X7" t="n">
-        <v>2312</v>
+        <v>2314</v>
       </c>
       <c r="Y7" t="n">
-        <v>5.9038</v>
+        <v>36.4114</v>
       </c>
       <c r="Z7" t="inlineStr">
         <is>
@@ -1204,7 +1225,7 @@
       </c>
       <c r="AG7" t="inlineStr">
         <is>
-          <t>FALSE</t>
+          <t>TRUE</t>
         </is>
       </c>
       <c r="AH7" t="inlineStr">
@@ -1214,39 +1235,39 @@
       </c>
       <c r="AI7" t="inlineStr">
         <is>
-          <t>TP</t>
+          <t>SL</t>
         </is>
       </c>
       <c r="AJ7" t="n">
-        <v>29545</v>
+        <v>27228.75</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>2026-05-15</t>
+          <t>2026-04-27</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>29241.25</v>
+        <v>27363.75</v>
       </c>
       <c r="C8" t="n">
-        <v>29291.25</v>
+        <v>27435</v>
       </c>
       <c r="D8" t="n">
-        <v>200</v>
+        <v>285</v>
       </c>
       <c r="E8" t="n">
-        <v>29294.96</v>
+        <v>27430.76</v>
       </c>
       <c r="F8" t="n">
-        <v>10</v>
+        <v>35</v>
       </c>
       <c r="G8" t="n">
-        <v>367</v>
+        <v>843</v>
       </c>
       <c r="H8" t="n">
-        <v>-145</v>
+        <v>-169</v>
       </c>
       <c r="I8" t="inlineStr">
         <is>
@@ -1254,19 +1275,19 @@
         </is>
       </c>
       <c r="J8" t="n">
-        <v>4.64</v>
+        <v>2.01</v>
       </c>
       <c r="K8" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="L8" t="n">
-        <v>29253.75</v>
+        <v>27370</v>
       </c>
       <c r="M8" t="n">
-        <v>29238.75</v>
+        <v>27355</v>
       </c>
       <c r="N8" t="n">
-        <v>29208.75</v>
+        <v>27325</v>
       </c>
       <c r="O8" t="n">
         <v>60</v>
@@ -1274,8 +1295,8 @@
       <c r="P8" t="n">
         <v>120</v>
       </c>
-      <c r="Q8" s="4" t="n">
-        <v>120</v>
+      <c r="Q8" s="7" t="n">
+        <v>-60</v>
       </c>
       <c r="R8" t="inlineStr">
         <is>
@@ -1288,11 +1309,11 @@
         </is>
       </c>
       <c r="T8" t="n">
+        <v>60</v>
+      </c>
+      <c r="U8" t="n">
         <v>5</v>
       </c>
-      <c r="U8" t="n">
-        <v>130</v>
-      </c>
       <c r="V8" t="inlineStr">
         <is>
           <t>score-exporter-2026-05-25-fast-exit-half-mfe</t>
@@ -1300,14 +1321,14 @@
       </c>
       <c r="W8" t="inlineStr">
         <is>
-          <t>09:31:00</t>
+          <t>09:36:00</t>
         </is>
       </c>
       <c r="X8" t="n">
-        <v>2311</v>
+        <v>2316</v>
       </c>
       <c r="Y8" t="n">
-        <v>2.1573</v>
+        <v>17.4372</v>
       </c>
       <c r="Z8" t="inlineStr">
         <is>
@@ -1331,7 +1352,7 @@
       </c>
       <c r="AD8" t="inlineStr">
         <is>
-          <t>FALSE</t>
+          <t>TRUE</t>
         </is>
       </c>
       <c r="AE8" t="inlineStr">
@@ -1356,39 +1377,39 @@
       </c>
       <c r="AI8" t="inlineStr">
         <is>
-          <t>TP</t>
+          <t>SL</t>
         </is>
       </c>
       <c r="AJ8" t="n">
-        <v>29208.75</v>
+        <v>27370</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2026-05-18</t>
+          <t>2026-04-28</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>29305</v>
+        <v>27082.5</v>
       </c>
       <c r="C9" t="n">
-        <v>29356.25</v>
+        <v>27162.5</v>
       </c>
       <c r="D9" t="n">
-        <v>205</v>
+        <v>320</v>
       </c>
       <c r="E9" t="n">
-        <v>29211.89</v>
+        <v>27189.12</v>
       </c>
       <c r="F9" t="n">
-        <v>60</v>
+        <v>50</v>
       </c>
       <c r="G9" t="n">
-        <v>800</v>
+        <v>957</v>
       </c>
       <c r="H9" t="n">
-        <v>-160</v>
+        <v>127</v>
       </c>
       <c r="I9" t="inlineStr">
         <is>
@@ -1396,19 +1417,19 @@
         </is>
       </c>
       <c r="J9" t="n">
-        <v>4.69</v>
+        <v>2.12</v>
       </c>
       <c r="K9" t="n">
         <v>5</v>
       </c>
       <c r="L9" t="n">
-        <v>29296.25</v>
+        <v>27168.75</v>
       </c>
       <c r="M9" t="n">
-        <v>29281.25</v>
+        <v>27183.75</v>
       </c>
       <c r="N9" t="n">
-        <v>29251.25</v>
+        <v>27213.75</v>
       </c>
       <c r="O9" t="n">
         <v>60</v>
@@ -1416,24 +1437,24 @@
       <c r="P9" t="n">
         <v>120</v>
       </c>
-      <c r="Q9" s="4" t="n">
+      <c r="Q9" s="7" t="n">
         <v>-60</v>
       </c>
       <c r="R9" t="inlineStr">
         <is>
-          <t>SELL</t>
+          <t>BUY</t>
         </is>
       </c>
       <c r="S9" t="inlineStr">
         <is>
-          <t>SELL1</t>
+          <t>BUY1</t>
         </is>
       </c>
       <c r="T9" t="n">
         <v>60</v>
       </c>
       <c r="U9" t="n">
-        <v>0</v>
+        <v>15</v>
       </c>
       <c r="V9" t="inlineStr">
         <is>
@@ -1442,14 +1463,14 @@
       </c>
       <c r="W9" t="inlineStr">
         <is>
-          <t>09:33:00</t>
+          <t>09:38:00</t>
         </is>
       </c>
       <c r="X9" t="n">
-        <v>2313</v>
+        <v>2318</v>
       </c>
       <c r="Y9" t="n">
-        <v>12.781</v>
+        <v>23.5896</v>
       </c>
       <c r="Z9" t="inlineStr">
         <is>
@@ -1502,35 +1523,35 @@
         </is>
       </c>
       <c r="AJ9" t="n">
-        <v>29296.25</v>
+        <v>27168.75</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>2026-05-19</t>
+          <t>2026-04-29</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>28851.25</v>
+        <v>27151.25</v>
       </c>
       <c r="C10" t="n">
-        <v>28943.75</v>
+        <v>27218.75</v>
       </c>
       <c r="D10" t="n">
-        <v>370</v>
+        <v>270</v>
       </c>
       <c r="E10" t="n">
-        <v>28925.07</v>
+        <v>27241.75</v>
       </c>
       <c r="F10" t="n">
-        <v>20</v>
+        <v>15</v>
       </c>
       <c r="G10" t="n">
-        <v>388</v>
+        <v>806</v>
       </c>
       <c r="H10" t="n">
-        <v>32</v>
+        <v>-88</v>
       </c>
       <c r="I10" t="inlineStr">
         <is>
@@ -1538,19 +1559,19 @@
         </is>
       </c>
       <c r="J10" t="n">
-        <v>3.64</v>
+        <v>2.3</v>
       </c>
       <c r="K10" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="L10" t="n">
-        <v>28933.75</v>
+        <v>27162.5</v>
       </c>
       <c r="M10" t="n">
-        <v>28948.75</v>
+        <v>27147.5</v>
       </c>
       <c r="N10" t="n">
-        <v>28978.75</v>
+        <v>27117.5</v>
       </c>
       <c r="O10" t="n">
         <v>60</v>
@@ -1558,24 +1579,24 @@
       <c r="P10" t="n">
         <v>120</v>
       </c>
-      <c r="Q10" s="4" t="n">
-        <v>120</v>
+      <c r="Q10" s="7" t="n">
+        <v>20</v>
       </c>
       <c r="R10" t="inlineStr">
         <is>
-          <t>BUY</t>
+          <t>SELL</t>
         </is>
       </c>
       <c r="S10" t="inlineStr">
         <is>
-          <t>BUY1</t>
+          <t>SELL1</t>
         </is>
       </c>
       <c r="T10" t="n">
-        <v>25</v>
+        <v>0</v>
       </c>
       <c r="U10" t="n">
-        <v>125</v>
+        <v>40</v>
       </c>
       <c r="V10" t="inlineStr">
         <is>
@@ -1584,14 +1605,14 @@
       </c>
       <c r="W10" t="inlineStr">
         <is>
-          <t>09:32:00</t>
+          <t>09:31:00</t>
         </is>
       </c>
       <c r="X10" t="n">
-        <v>2312</v>
+        <v>2311</v>
       </c>
       <c r="Y10" t="n">
-        <v>5.4978</v>
+        <v>6.5119</v>
       </c>
       <c r="Z10" t="inlineStr">
         <is>
@@ -1605,7 +1626,7 @@
       </c>
       <c r="AB10" t="inlineStr">
         <is>
-          <t>FALSE</t>
+          <t>TRUE</t>
         </is>
       </c>
       <c r="AC10" t="inlineStr">
@@ -1615,7 +1636,7 @@
       </c>
       <c r="AD10" t="inlineStr">
         <is>
-          <t>FALSE</t>
+          <t>TRUE</t>
         </is>
       </c>
       <c r="AE10" t="inlineStr">
@@ -1640,39 +1661,39 @@
       </c>
       <c r="AI10" t="inlineStr">
         <is>
-          <t>TP</t>
+          <t>EXIT</t>
         </is>
       </c>
       <c r="AJ10" t="n">
-        <v>28978.75</v>
+        <v>27142.5</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-04-30</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>29070</v>
+        <v>27422.5</v>
       </c>
       <c r="C11" t="n">
-        <v>29122.5</v>
+        <v>27492.5</v>
       </c>
       <c r="D11" t="n">
-        <v>210</v>
+        <v>280</v>
       </c>
       <c r="E11" t="n">
-        <v>29074.59</v>
-      </c>
-      <c r="F11" t="n">
-        <v>25</v>
+        <v>27385.42</v>
+      </c>
+      <c r="F11" s="5" t="n">
+        <v>30</v>
       </c>
       <c r="G11" t="n">
-        <v>1130</v>
+        <v>984</v>
       </c>
       <c r="H11" t="n">
-        <v>184</v>
+        <v>-110</v>
       </c>
       <c r="I11" t="inlineStr">
         <is>
@@ -1680,19 +1701,19 @@
         </is>
       </c>
       <c r="J11" t="n">
-        <v>3.1</v>
+        <v>2.55</v>
       </c>
       <c r="K11" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="L11" t="n">
-        <v>29113.75</v>
+        <v>27430</v>
       </c>
       <c r="M11" t="n">
-        <v>29128.75</v>
+        <v>27415</v>
       </c>
       <c r="N11" t="n">
-        <v>29158.75</v>
+        <v>27385</v>
       </c>
       <c r="O11" t="n">
         <v>60</v>
@@ -1700,24 +1721,24 @@
       <c r="P11" t="n">
         <v>120</v>
       </c>
-      <c r="Q11" s="4" t="n">
-        <v>-60</v>
+      <c r="Q11" s="7" t="n">
+        <v>22.5</v>
       </c>
       <c r="R11" t="inlineStr">
         <is>
-          <t>BUY</t>
+          <t>SELL</t>
         </is>
       </c>
       <c r="S11" t="inlineStr">
         <is>
-          <t>BUY1</t>
+          <t>SELL1</t>
         </is>
       </c>
       <c r="T11" t="n">
-        <v>60</v>
+        <v>50</v>
       </c>
       <c r="U11" t="n">
-        <v>30</v>
+        <v>45</v>
       </c>
       <c r="V11" t="inlineStr">
         <is>
@@ -1733,7 +1754,7 @@
         <v>2311</v>
       </c>
       <c r="Y11" t="n">
-        <v>8.0563</v>
+        <v>11.7789</v>
       </c>
       <c r="Z11" t="inlineStr">
         <is>
@@ -1772,7 +1793,7 @@
       </c>
       <c r="AG11" t="inlineStr">
         <is>
-          <t>TRUE</t>
+          <t>FALSE</t>
         </is>
       </c>
       <c r="AH11" t="inlineStr">
@@ -1782,84 +1803,84 @@
       </c>
       <c r="AI11" t="inlineStr">
         <is>
-          <t>SL</t>
+          <t>EXIT</t>
         </is>
       </c>
       <c r="AJ11" t="n">
-        <v>29113.75</v>
+        <v>27409.38</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-01</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>29193.75</v>
+        <v>27618.75</v>
       </c>
       <c r="C12" t="n">
-        <v>29250</v>
+        <v>27666.25</v>
       </c>
       <c r="D12" t="n">
-        <v>225</v>
+        <v>190</v>
       </c>
       <c r="E12" t="n">
-        <v>29289.99</v>
+        <v>27598.29</v>
       </c>
       <c r="F12" t="n">
-        <v>50</v>
+        <v>25</v>
       </c>
       <c r="G12" t="n">
-        <v>183</v>
+        <v>825</v>
       </c>
       <c r="H12" t="n">
-        <v>-63</v>
+        <v>247</v>
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>A+ speed</t>
+          <t>normal speed</t>
         </is>
       </c>
       <c r="J12" t="n">
-        <v>302.19</v>
+        <v>3.29</v>
       </c>
       <c r="K12" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="L12" t="n">
-        <v>29206.25</v>
+        <v>27657.5</v>
       </c>
       <c r="M12" t="n">
-        <v>29181.25</v>
+        <v>27672.5</v>
       </c>
       <c r="N12" t="n">
-        <v>29151.25</v>
+        <v>27702.5</v>
       </c>
       <c r="O12" t="n">
-        <v>100</v>
+        <v>60</v>
       </c>
       <c r="P12" t="n">
         <v>120</v>
       </c>
-      <c r="Q12" s="4" t="n">
-        <v>-100</v>
+      <c r="Q12" s="7" t="n">
+        <v>52.5</v>
       </c>
       <c r="R12" t="inlineStr">
         <is>
-          <t>SELL</t>
+          <t>BUY</t>
         </is>
       </c>
       <c r="S12" t="inlineStr">
         <is>
-          <t>SELL</t>
+          <t>BUY1</t>
         </is>
       </c>
       <c r="T12" t="n">
+        <v>5</v>
+      </c>
+      <c r="U12" t="n">
         <v>105</v>
-      </c>
-      <c r="U12" t="n">
-        <v>0</v>
       </c>
       <c r="V12" t="inlineStr">
         <is>
@@ -1875,7 +1896,7 @@
         <v>2311</v>
       </c>
       <c r="Y12" t="n">
-        <v>0.1655</v>
+        <v>7.5947</v>
       </c>
       <c r="Z12" t="inlineStr">
         <is>
@@ -1899,7 +1920,7 @@
       </c>
       <c r="AD12" t="inlineStr">
         <is>
-          <t>FALSE</t>
+          <t>TRUE</t>
         </is>
       </c>
       <c r="AE12" t="inlineStr">
@@ -1924,39 +1945,39 @@
       </c>
       <c r="AI12" t="inlineStr">
         <is>
-          <t>SL</t>
+          <t>EXIT</t>
         </is>
       </c>
       <c r="AJ12" t="n">
-        <v>29206.25</v>
+        <v>27685.63</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>2026-05-22</t>
+          <t>2026-05-04</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>29551.25</v>
+        <v>27837.5</v>
       </c>
       <c r="C13" t="n">
-        <v>29620</v>
+        <v>27875</v>
       </c>
       <c r="D13" t="n">
-        <v>275</v>
+        <v>150</v>
       </c>
       <c r="E13" t="n">
-        <v>29557.5</v>
+        <v>27837.01</v>
       </c>
       <c r="F13" t="n">
-        <v>25</v>
+        <v>40</v>
       </c>
       <c r="G13" t="n">
-        <v>812</v>
+        <v>1327</v>
       </c>
       <c r="H13" t="n">
-        <v>-8</v>
+        <v>-23</v>
       </c>
       <c r="I13" t="inlineStr">
         <is>
@@ -1964,19 +1985,19 @@
         </is>
       </c>
       <c r="J13" t="n">
-        <v>3.2</v>
+        <v>2.25</v>
       </c>
       <c r="K13" t="n">
         <v>6</v>
       </c>
       <c r="L13" t="n">
-        <v>29611.25</v>
+        <v>27842.5</v>
       </c>
       <c r="M13" t="n">
-        <v>29626.25</v>
+        <v>27827.5</v>
       </c>
       <c r="N13" t="n">
-        <v>29656.25</v>
+        <v>27797.5</v>
       </c>
       <c r="O13" t="n">
         <v>60</v>
@@ -1984,24 +2005,24 @@
       <c r="P13" t="n">
         <v>120</v>
       </c>
-      <c r="Q13" s="4" t="n">
-        <v>22.5</v>
+      <c r="Q13" s="7" t="n">
+        <v>35</v>
       </c>
       <c r="R13" t="inlineStr">
         <is>
-          <t>BUY</t>
+          <t>SELL</t>
         </is>
       </c>
       <c r="S13" t="inlineStr">
         <is>
-          <t>BUY1</t>
+          <t>SELL1</t>
         </is>
       </c>
       <c r="T13" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="U13" t="n">
-        <v>45</v>
+        <v>70</v>
       </c>
       <c r="V13" t="inlineStr">
         <is>
@@ -2017,7 +2038,7 @@
         <v>2311</v>
       </c>
       <c r="Y13" t="n">
-        <v>7.8201</v>
+        <v>17.7523</v>
       </c>
       <c r="Z13" t="inlineStr">
         <is>
@@ -2070,10 +2091,1857 @@
         </is>
       </c>
       <c r="AJ13" t="n">
-        <v>29631.88</v>
+        <v>27818.75</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>2026-05-05</t>
+        </is>
+      </c>
+      <c r="B14" t="n">
+        <v>27986.25</v>
+      </c>
+      <c r="C14" t="n">
+        <v>28023.75</v>
+      </c>
+      <c r="D14" t="n">
+        <v>150</v>
+      </c>
+      <c r="E14" t="n">
+        <v>27935.7</v>
+      </c>
+      <c r="F14" t="n">
+        <v>15</v>
+      </c>
+      <c r="G14" t="n">
+        <v>829</v>
+      </c>
+      <c r="H14" t="n">
+        <v>-135</v>
+      </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>normal speed</t>
+        </is>
+      </c>
+      <c r="J14" t="n">
+        <v>2.83</v>
+      </c>
+      <c r="K14" t="n">
+        <v>5</v>
+      </c>
+      <c r="L14" t="n">
+        <v>27997.5</v>
+      </c>
+      <c r="M14" t="n">
+        <v>27982.5</v>
+      </c>
+      <c r="N14" t="n">
+        <v>27952.5</v>
+      </c>
+      <c r="O14" t="n">
+        <v>60</v>
+      </c>
+      <c r="P14" t="n">
+        <v>120</v>
+      </c>
+      <c r="Q14" s="7" t="n">
+        <v>22.5</v>
+      </c>
+      <c r="R14" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="S14" t="inlineStr">
+        <is>
+          <t>SELL1</t>
+        </is>
+      </c>
+      <c r="T14" t="n">
+        <v>0</v>
+      </c>
+      <c r="U14" t="n">
+        <v>45</v>
+      </c>
+      <c r="V14" t="inlineStr">
+        <is>
+          <t>score-exporter-2026-05-25-fast-exit-half-mfe</t>
+        </is>
+      </c>
+      <c r="W14" t="inlineStr">
+        <is>
+          <t>09:31:00</t>
+        </is>
+      </c>
+      <c r="X14" t="n">
+        <v>2310</v>
+      </c>
+      <c r="Y14" t="n">
+        <v>5.3047</v>
+      </c>
+      <c r="Z14" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="AA14" t="inlineStr">
+        <is>
+          <t>LastTime</t>
+        </is>
+      </c>
+      <c r="AB14" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AC14" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AD14" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AE14" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AF14" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AG14" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="AH14" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AI14" t="inlineStr">
+        <is>
+          <t>EXIT</t>
+        </is>
+      </c>
+      <c r="AJ14" t="n">
+        <v>27976.88</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>2026-05-06</t>
+        </is>
+      </c>
+      <c r="B15" t="n">
+        <v>28336.25</v>
+      </c>
+      <c r="C15" t="n">
+        <v>28392.5</v>
+      </c>
+      <c r="D15" t="n">
+        <v>225</v>
+      </c>
+      <c r="E15" t="n">
+        <v>28455.83</v>
+      </c>
+      <c r="F15" t="n">
+        <v>25</v>
+      </c>
+      <c r="G15" t="n">
+        <v>835</v>
+      </c>
+      <c r="H15" t="n">
+        <v>27</v>
+      </c>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>normal speed</t>
+        </is>
+      </c>
+      <c r="J15" t="n">
+        <v>2.13</v>
+      </c>
+      <c r="K15" t="n">
+        <v>5</v>
+      </c>
+      <c r="L15" t="n">
+        <v>28411.25</v>
+      </c>
+      <c r="M15" t="n">
+        <v>28426.25</v>
+      </c>
+      <c r="N15" t="n">
+        <v>28456.25</v>
+      </c>
+      <c r="O15" t="n">
+        <v>60</v>
+      </c>
+      <c r="P15" t="n">
+        <v>120</v>
+      </c>
+      <c r="Q15" s="7" t="n">
+        <v>-60</v>
+      </c>
+      <c r="R15" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="S15" t="inlineStr">
+        <is>
+          <t>BUY1</t>
+        </is>
+      </c>
+      <c r="T15" t="n">
+        <v>60</v>
+      </c>
+      <c r="U15" t="n">
+        <v>0</v>
+      </c>
+      <c r="V15" t="inlineStr">
+        <is>
+          <t>score-exporter-2026-05-25-fast-exit-half-mfe</t>
+        </is>
+      </c>
+      <c r="W15" t="inlineStr">
+        <is>
+          <t>09:33:00</t>
+        </is>
+      </c>
+      <c r="X15" t="n">
+        <v>2313</v>
+      </c>
+      <c r="Y15" t="n">
+        <v>11.7309</v>
+      </c>
+      <c r="Z15" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="AA15" t="inlineStr">
+        <is>
+          <t>LastTime</t>
+        </is>
+      </c>
+      <c r="AB15" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AC15" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AD15" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AE15" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AF15" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AG15" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="AH15" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AI15" t="inlineStr">
+        <is>
+          <t>SL</t>
+        </is>
+      </c>
+      <c r="AJ15" t="n">
+        <v>28411.25</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>2026-05-07</t>
+        </is>
+      </c>
+      <c r="B16" t="n">
+        <v>28730</v>
+      </c>
+      <c r="C16" t="n">
+        <v>28766.25</v>
+      </c>
+      <c r="D16" t="n">
+        <v>145</v>
+      </c>
+      <c r="E16" t="n">
+        <v>28745.29</v>
+      </c>
+      <c r="F16" t="n">
+        <v>30</v>
+      </c>
+      <c r="G16" t="n">
+        <v>802</v>
+      </c>
+      <c r="H16" t="n">
+        <v>210</v>
+      </c>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>normal speed</t>
+        </is>
+      </c>
+      <c r="J16" t="n">
+        <v>4.17</v>
+      </c>
+      <c r="K16" t="n">
+        <v>7</v>
+      </c>
+      <c r="L16" t="n">
+        <v>28780</v>
+      </c>
+      <c r="M16" t="n">
+        <v>28795</v>
+      </c>
+      <c r="N16" t="n">
+        <v>28825</v>
+      </c>
+      <c r="O16" t="n">
+        <v>60</v>
+      </c>
+      <c r="P16" t="n">
+        <v>120</v>
+      </c>
+      <c r="Q16" s="7" t="n">
+        <v>-60</v>
+      </c>
+      <c r="R16" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="S16" t="inlineStr">
+        <is>
+          <t>BUY1</t>
+        </is>
+      </c>
+      <c r="T16" t="n">
+        <v>75</v>
+      </c>
+      <c r="U16" t="n">
+        <v>35</v>
+      </c>
+      <c r="V16" t="inlineStr">
+        <is>
+          <t>score-exporter-2026-05-25-fast-exit-half-mfe</t>
+        </is>
+      </c>
+      <c r="W16" t="inlineStr">
+        <is>
+          <t>09:55:00</t>
+        </is>
+      </c>
+      <c r="X16" t="n">
+        <v>2335</v>
+      </c>
+      <c r="Y16" t="n">
+        <v>7.1896</v>
+      </c>
+      <c r="Z16" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="AA16" t="inlineStr">
+        <is>
+          <t>LastTime</t>
+        </is>
+      </c>
+      <c r="AB16" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AC16" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AD16" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AE16" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AF16" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AG16" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AH16" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AI16" t="inlineStr">
+        <is>
+          <t>SL</t>
+        </is>
+      </c>
+      <c r="AJ16" t="n">
+        <v>28780</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>2026-05-08</t>
+        </is>
+      </c>
+      <c r="B17" t="n">
+        <v>28860</v>
+      </c>
+      <c r="C17" t="n">
+        <v>28903.75</v>
+      </c>
+      <c r="D17" t="n">
+        <v>175</v>
+      </c>
+      <c r="E17" t="n">
+        <v>28876.61</v>
+      </c>
+      <c r="F17" t="n">
+        <v>55</v>
+      </c>
+      <c r="G17" t="n">
+        <v>1578</v>
+      </c>
+      <c r="H17" t="n">
+        <v>210</v>
+      </c>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>normal speed</t>
+        </is>
+      </c>
+      <c r="J17" t="n">
+        <v>2.4</v>
+      </c>
+      <c r="K17" t="n">
+        <v>7</v>
+      </c>
+      <c r="L17" t="n">
+        <v>28902.5</v>
+      </c>
+      <c r="M17" t="n">
+        <v>28917.5</v>
+      </c>
+      <c r="N17" t="n">
+        <v>28947.5</v>
+      </c>
+      <c r="O17" t="n">
+        <v>60</v>
+      </c>
+      <c r="P17" t="n">
+        <v>120</v>
+      </c>
+      <c r="Q17" s="7" t="n">
+        <v>25</v>
+      </c>
+      <c r="R17" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="S17" t="inlineStr">
+        <is>
+          <t>BUY1</t>
+        </is>
+      </c>
+      <c r="T17" t="n">
+        <v>50</v>
+      </c>
+      <c r="U17" t="n">
+        <v>50</v>
+      </c>
+      <c r="V17" t="inlineStr">
+        <is>
+          <t>score-exporter-2026-05-25-fast-exit-half-mfe</t>
+        </is>
+      </c>
+      <c r="W17" t="inlineStr">
+        <is>
+          <t>09:31:00</t>
+        </is>
+      </c>
+      <c r="X17" t="n">
+        <v>2311</v>
+      </c>
+      <c r="Y17" t="n">
+        <v>22.9295</v>
+      </c>
+      <c r="Z17" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="AA17" t="inlineStr">
+        <is>
+          <t>LastTime</t>
+        </is>
+      </c>
+      <c r="AB17" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AC17" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AD17" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AE17" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AF17" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AG17" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AH17" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AI17" t="inlineStr">
+        <is>
+          <t>EXIT</t>
+        </is>
+      </c>
+      <c r="AJ17" t="n">
+        <v>28923.75</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>2026-05-11</t>
+        </is>
+      </c>
+      <c r="B18" t="n">
+        <v>29282.5</v>
+      </c>
+      <c r="C18" t="n">
+        <v>29346.25</v>
+      </c>
+      <c r="D18" t="n">
+        <v>255</v>
+      </c>
+      <c r="E18" t="n">
+        <v>29316.62</v>
+      </c>
+      <c r="F18" t="n">
+        <v>75</v>
+      </c>
+      <c r="G18" t="n">
+        <v>816</v>
+      </c>
+      <c r="H18" t="n">
+        <v>138</v>
+      </c>
+      <c r="I18" t="inlineStr">
+        <is>
+          <t>A+ speed</t>
+        </is>
+      </c>
+      <c r="J18" t="n">
+        <v>10.7</v>
+      </c>
+      <c r="K18" t="n">
+        <v>7</v>
+      </c>
+      <c r="L18" t="n">
+        <v>29340</v>
+      </c>
+      <c r="M18" t="n">
+        <v>29365</v>
+      </c>
+      <c r="N18" t="n">
+        <v>29395</v>
+      </c>
+      <c r="O18" t="n">
+        <v>100</v>
+      </c>
+      <c r="P18" t="n">
+        <v>120</v>
+      </c>
+      <c r="Q18" s="7" t="n">
+        <v>120</v>
+      </c>
+      <c r="R18" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="S18" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="T18" t="n">
+        <v>15</v>
+      </c>
+      <c r="U18" t="n">
+        <v>120</v>
+      </c>
+      <c r="V18" t="inlineStr">
+        <is>
+          <t>score-exporter-2026-05-25-fast-exit-half-mfe</t>
+        </is>
+      </c>
+      <c r="W18" t="inlineStr">
+        <is>
+          <t>09:31:00</t>
+        </is>
+      </c>
+      <c r="X18" t="n">
+        <v>2311</v>
+      </c>
+      <c r="Y18" t="n">
+        <v>7.0112</v>
+      </c>
+      <c r="Z18" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="AA18" t="inlineStr">
+        <is>
+          <t>LastTime</t>
+        </is>
+      </c>
+      <c r="AB18" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AC18" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AD18" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AE18" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AF18" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AG18" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AH18" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AI18" t="inlineStr">
+        <is>
+          <t>TP</t>
+        </is>
+      </c>
+      <c r="AJ18" t="n">
+        <v>29395</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>2026-05-12</t>
+        </is>
+      </c>
+      <c r="B19" t="n">
+        <v>29146.25</v>
+      </c>
+      <c r="C19" t="n">
+        <v>29227.5</v>
+      </c>
+      <c r="D19" t="n">
+        <v>325</v>
+      </c>
+      <c r="E19" t="n">
+        <v>29203.6</v>
+      </c>
+      <c r="F19" t="n">
+        <v>35</v>
+      </c>
+      <c r="G19" t="n">
+        <v>801</v>
+      </c>
+      <c r="H19" t="n">
+        <v>97</v>
+      </c>
+      <c r="I19" t="inlineStr">
+        <is>
+          <t>normal speed</t>
+        </is>
+      </c>
+      <c r="J19" t="n">
+        <v>2.98</v>
+      </c>
+      <c r="K19" t="n">
+        <v>7</v>
+      </c>
+      <c r="L19" t="n">
+        <v>29231.25</v>
+      </c>
+      <c r="M19" t="n">
+        <v>29246.25</v>
+      </c>
+      <c r="N19" t="n">
+        <v>29276.25</v>
+      </c>
+      <c r="O19" t="n">
+        <v>60</v>
+      </c>
+      <c r="P19" t="n">
+        <v>120</v>
+      </c>
+      <c r="Q19" s="7" t="n">
+        <v>-60</v>
+      </c>
+      <c r="R19" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="S19" t="inlineStr">
+        <is>
+          <t>BUY1</t>
+        </is>
+      </c>
+      <c r="T19" t="n">
+        <v>60</v>
+      </c>
+      <c r="U19" t="n">
+        <v>5</v>
+      </c>
+      <c r="V19" t="inlineStr">
+        <is>
+          <t>score-exporter-2026-05-25-fast-exit-half-mfe</t>
+        </is>
+      </c>
+      <c r="W19" t="inlineStr">
+        <is>
+          <t>09:41:00</t>
+        </is>
+      </c>
+      <c r="X19" t="n">
+        <v>2321</v>
+      </c>
+      <c r="Y19" t="n">
+        <v>11.7355</v>
+      </c>
+      <c r="Z19" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="AA19" t="inlineStr">
+        <is>
+          <t>LastTime</t>
+        </is>
+      </c>
+      <c r="AB19" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AC19" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AD19" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AE19" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AF19" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AG19" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AH19" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AI19" t="inlineStr">
+        <is>
+          <t>SL</t>
+        </is>
+      </c>
+      <c r="AJ19" t="n">
+        <v>29231.25</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>2026-05-13</t>
+        </is>
+      </c>
+      <c r="B20" t="n">
+        <v>29252.5</v>
+      </c>
+      <c r="C20" t="n">
+        <v>29288.75</v>
+      </c>
+      <c r="D20" t="n">
+        <v>145</v>
+      </c>
+      <c r="E20" t="n">
+        <v>29321.35</v>
+      </c>
+      <c r="F20" t="n">
+        <v>40</v>
+      </c>
+      <c r="G20" t="n">
+        <v>1126</v>
+      </c>
+      <c r="H20" t="n">
+        <v>-176</v>
+      </c>
+      <c r="I20" t="inlineStr">
+        <is>
+          <t>normal speed</t>
+        </is>
+      </c>
+      <c r="J20" t="n">
+        <v>2.37</v>
+      </c>
+      <c r="K20" t="n">
+        <v>7</v>
+      </c>
+      <c r="L20" t="n">
+        <v>29257.5</v>
+      </c>
+      <c r="M20" t="n">
+        <v>29242.5</v>
+      </c>
+      <c r="N20" t="n">
+        <v>29212.5</v>
+      </c>
+      <c r="O20" t="n">
+        <v>60</v>
+      </c>
+      <c r="P20" t="n">
+        <v>120</v>
+      </c>
+      <c r="Q20" s="7" t="n">
+        <v>27.5</v>
+      </c>
+      <c r="R20" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="S20" t="inlineStr">
+        <is>
+          <t>SELL1</t>
+        </is>
+      </c>
+      <c r="T20" t="n">
+        <v>5</v>
+      </c>
+      <c r="U20" t="n">
+        <v>55</v>
+      </c>
+      <c r="V20" t="inlineStr">
+        <is>
+          <t>score-exporter-2026-05-25-fast-exit-half-mfe</t>
+        </is>
+      </c>
+      <c r="W20" t="inlineStr">
+        <is>
+          <t>09:31:00</t>
+        </is>
+      </c>
+      <c r="X20" t="n">
+        <v>2311</v>
+      </c>
+      <c r="Y20" t="n">
+        <v>16.8754</v>
+      </c>
+      <c r="Z20" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="AA20" t="inlineStr">
+        <is>
+          <t>LastTime</t>
+        </is>
+      </c>
+      <c r="AB20" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AC20" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AD20" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AE20" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AF20" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AG20" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AH20" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AI20" t="inlineStr">
+        <is>
+          <t>EXIT</t>
+        </is>
+      </c>
+      <c r="AJ20" t="n">
+        <v>29235.63</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>2026-05-14</t>
+        </is>
+      </c>
+      <c r="B21" t="n">
+        <v>29460</v>
+      </c>
+      <c r="C21" t="n">
+        <v>29492.5</v>
+      </c>
+      <c r="D21" t="n">
+        <v>130</v>
+      </c>
+      <c r="E21" t="n">
+        <v>29543.51</v>
+      </c>
+      <c r="F21" t="n">
+        <v>65</v>
+      </c>
+      <c r="G21" t="n">
+        <v>801</v>
+      </c>
+      <c r="H21" t="n">
+        <v>263</v>
+      </c>
+      <c r="I21" t="inlineStr">
+        <is>
+          <t>A+ speed</t>
+        </is>
+      </c>
+      <c r="J21" t="n">
+        <v>11.01</v>
+      </c>
+      <c r="K21" t="n">
+        <v>5</v>
+      </c>
+      <c r="L21" t="n">
+        <v>29490</v>
+      </c>
+      <c r="M21" t="n">
+        <v>29515</v>
+      </c>
+      <c r="N21" t="n">
+        <v>29545</v>
+      </c>
+      <c r="O21" t="n">
+        <v>100</v>
+      </c>
+      <c r="P21" t="n">
+        <v>120</v>
+      </c>
+      <c r="Q21" s="7" t="n">
+        <v>120</v>
+      </c>
+      <c r="R21" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="S21" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="T21" t="n">
+        <v>25</v>
+      </c>
+      <c r="U21" t="n">
+        <v>120</v>
+      </c>
+      <c r="V21" t="inlineStr">
+        <is>
+          <t>score-exporter-2026-05-25-fast-exit-half-mfe</t>
+        </is>
+      </c>
+      <c r="W21" t="inlineStr">
+        <is>
+          <t>09:32:00</t>
+        </is>
+      </c>
+      <c r="X21" t="n">
+        <v>2312</v>
+      </c>
+      <c r="Y21" t="n">
+        <v>5.9038</v>
+      </c>
+      <c r="Z21" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="AA21" t="inlineStr">
+        <is>
+          <t>LastTime</t>
+        </is>
+      </c>
+      <c r="AB21" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AC21" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AD21" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AE21" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AF21" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AG21" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="AH21" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AI21" t="inlineStr">
+        <is>
+          <t>TP</t>
+        </is>
+      </c>
+      <c r="AJ21" t="n">
+        <v>29545</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>2026-05-15</t>
+        </is>
+      </c>
+      <c r="B22" t="n">
+        <v>29241.25</v>
+      </c>
+      <c r="C22" t="n">
+        <v>29291.25</v>
+      </c>
+      <c r="D22" t="n">
+        <v>200</v>
+      </c>
+      <c r="E22" t="n">
+        <v>29294.78</v>
+      </c>
+      <c r="F22" t="n">
+        <v>90</v>
+      </c>
+      <c r="G22" t="n">
+        <v>814</v>
+      </c>
+      <c r="H22" t="n">
+        <v>-358</v>
+      </c>
+      <c r="I22" t="inlineStr">
+        <is>
+          <t>A+ speed</t>
+        </is>
+      </c>
+      <c r="J22" t="n">
+        <v>18.05</v>
+      </c>
+      <c r="K22" t="n">
+        <v>7</v>
+      </c>
+      <c r="L22" t="n">
+        <v>29243.75</v>
+      </c>
+      <c r="M22" t="n">
+        <v>29218.75</v>
+      </c>
+      <c r="N22" t="n">
+        <v>29188.75</v>
+      </c>
+      <c r="O22" t="n">
+        <v>100</v>
+      </c>
+      <c r="P22" t="n">
+        <v>120</v>
+      </c>
+      <c r="Q22" s="7" t="n">
+        <v>-100</v>
+      </c>
+      <c r="R22" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="S22" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="T22" t="n">
+        <v>100</v>
+      </c>
+      <c r="U22" t="n">
+        <v>60</v>
+      </c>
+      <c r="V22" t="inlineStr">
+        <is>
+          <t>score-exporter-2026-05-25-fast-exit-half-mfe</t>
+        </is>
+      </c>
+      <c r="W22" t="inlineStr">
+        <is>
+          <t>09:31:00</t>
+        </is>
+      </c>
+      <c r="X22" t="n">
+        <v>2311</v>
+      </c>
+      <c r="Y22" t="n">
+        <v>4.9856</v>
+      </c>
+      <c r="Z22" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="AA22" t="inlineStr">
+        <is>
+          <t>LastTime</t>
+        </is>
+      </c>
+      <c r="AB22" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AC22" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AD22" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AE22" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AF22" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AG22" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AH22" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AI22" t="inlineStr">
+        <is>
+          <t>SL</t>
+        </is>
+      </c>
+      <c r="AJ22" t="n">
+        <v>29243.75</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>2026-05-18</t>
+        </is>
+      </c>
+      <c r="B23" t="n">
+        <v>29305</v>
+      </c>
+      <c r="C23" t="n">
+        <v>29356.25</v>
+      </c>
+      <c r="D23" t="n">
+        <v>205</v>
+      </c>
+      <c r="E23" t="n">
+        <v>29211.89</v>
+      </c>
+      <c r="F23" t="n">
+        <v>60</v>
+      </c>
+      <c r="G23" t="n">
+        <v>800</v>
+      </c>
+      <c r="H23" t="n">
+        <v>-160</v>
+      </c>
+      <c r="I23" t="inlineStr">
+        <is>
+          <t>normal speed</t>
+        </is>
+      </c>
+      <c r="J23" t="n">
+        <v>4.69</v>
+      </c>
+      <c r="K23" t="n">
+        <v>5</v>
+      </c>
+      <c r="L23" t="n">
+        <v>29296.25</v>
+      </c>
+      <c r="M23" t="n">
+        <v>29281.25</v>
+      </c>
+      <c r="N23" t="n">
+        <v>29251.25</v>
+      </c>
+      <c r="O23" t="n">
+        <v>60</v>
+      </c>
+      <c r="P23" t="n">
+        <v>120</v>
+      </c>
+      <c r="Q23" s="7" t="n">
+        <v>-60</v>
+      </c>
+      <c r="R23" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="S23" t="inlineStr">
+        <is>
+          <t>SELL1</t>
+        </is>
+      </c>
+      <c r="T23" t="n">
+        <v>60</v>
+      </c>
+      <c r="U23" t="n">
+        <v>0</v>
+      </c>
+      <c r="V23" t="inlineStr">
+        <is>
+          <t>score-exporter-2026-05-25-fast-exit-half-mfe</t>
+        </is>
+      </c>
+      <c r="W23" t="inlineStr">
+        <is>
+          <t>09:33:00</t>
+        </is>
+      </c>
+      <c r="X23" t="n">
+        <v>2313</v>
+      </c>
+      <c r="Y23" t="n">
+        <v>12.781</v>
+      </c>
+      <c r="Z23" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="AA23" t="inlineStr">
+        <is>
+          <t>LastTime</t>
+        </is>
+      </c>
+      <c r="AB23" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AC23" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AD23" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AE23" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AF23" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AG23" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="AH23" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AI23" t="inlineStr">
+        <is>
+          <t>SL</t>
+        </is>
+      </c>
+      <c r="AJ23" t="n">
+        <v>29296.25</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>2026-05-19</t>
+        </is>
+      </c>
+      <c r="B24" t="n">
+        <v>28851.25</v>
+      </c>
+      <c r="C24" t="n">
+        <v>28943.75</v>
+      </c>
+      <c r="D24" t="n">
+        <v>370</v>
+      </c>
+      <c r="E24" t="n">
+        <v>28925.15</v>
+      </c>
+      <c r="F24" t="n">
+        <v>35</v>
+      </c>
+      <c r="G24" t="n">
+        <v>831</v>
+      </c>
+      <c r="H24" t="n">
+        <v>125</v>
+      </c>
+      <c r="I24" t="inlineStr">
+        <is>
+          <t>normal speed</t>
+        </is>
+      </c>
+      <c r="J24" t="n">
+        <v>2.39</v>
+      </c>
+      <c r="K24" t="n">
+        <v>6</v>
+      </c>
+      <c r="L24" t="n">
+        <v>28937.5</v>
+      </c>
+      <c r="M24" t="n">
+        <v>28952.5</v>
+      </c>
+      <c r="N24" t="n">
+        <v>28982.5</v>
+      </c>
+      <c r="O24" t="n">
+        <v>60</v>
+      </c>
+      <c r="P24" t="n">
+        <v>120</v>
+      </c>
+      <c r="Q24" s="7" t="n">
+        <v>120</v>
+      </c>
+      <c r="R24" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="S24" t="inlineStr">
+        <is>
+          <t>BUY1</t>
+        </is>
+      </c>
+      <c r="T24" t="n">
+        <v>0</v>
+      </c>
+      <c r="U24" t="n">
+        <v>120</v>
+      </c>
+      <c r="V24" t="inlineStr">
+        <is>
+          <t>score-exporter-2026-05-25-fast-exit-half-mfe</t>
+        </is>
+      </c>
+      <c r="W24" t="inlineStr">
+        <is>
+          <t>09:32:00</t>
+        </is>
+      </c>
+      <c r="X24" t="n">
+        <v>2312</v>
+      </c>
+      <c r="Y24" t="n">
+        <v>14.6523</v>
+      </c>
+      <c r="Z24" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="AA24" t="inlineStr">
+        <is>
+          <t>LastTime</t>
+        </is>
+      </c>
+      <c r="AB24" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="AC24" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AD24" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AE24" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AF24" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AG24" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AH24" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AI24" t="inlineStr">
+        <is>
+          <t>TP</t>
+        </is>
+      </c>
+      <c r="AJ24" t="n">
+        <v>28982.5</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>2026-05-20</t>
+        </is>
+      </c>
+      <c r="B25" t="n">
+        <v>29070</v>
+      </c>
+      <c r="C25" t="n">
+        <v>29122.5</v>
+      </c>
+      <c r="D25" t="n">
+        <v>210</v>
+      </c>
+      <c r="E25" t="n">
+        <v>29074.61</v>
+      </c>
+      <c r="F25" t="n">
+        <v>20</v>
+      </c>
+      <c r="G25" t="n">
+        <v>1184</v>
+      </c>
+      <c r="H25" t="n">
+        <v>198</v>
+      </c>
+      <c r="I25" t="inlineStr">
+        <is>
+          <t>normal speed</t>
+        </is>
+      </c>
+      <c r="J25" t="n">
+        <v>2.29</v>
+      </c>
+      <c r="K25" t="n">
+        <v>7</v>
+      </c>
+      <c r="L25" t="n">
+        <v>29112.5</v>
+      </c>
+      <c r="M25" t="n">
+        <v>29127.5</v>
+      </c>
+      <c r="N25" t="n">
+        <v>29157.5</v>
+      </c>
+      <c r="O25" t="n">
+        <v>60</v>
+      </c>
+      <c r="P25" t="n">
+        <v>120</v>
+      </c>
+      <c r="Q25" s="7" t="n">
+        <v>-60</v>
+      </c>
+      <c r="R25" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="S25" t="inlineStr">
+        <is>
+          <t>BUY1</t>
+        </is>
+      </c>
+      <c r="T25" t="n">
+        <v>60</v>
+      </c>
+      <c r="U25" t="n">
+        <v>35</v>
+      </c>
+      <c r="V25" t="inlineStr">
+        <is>
+          <t>score-exporter-2026-05-25-fast-exit-half-mfe</t>
+        </is>
+      </c>
+      <c r="W25" t="inlineStr">
+        <is>
+          <t>09:31:00</t>
+        </is>
+      </c>
+      <c r="X25" t="n">
+        <v>2311</v>
+      </c>
+      <c r="Y25" t="n">
+        <v>8.7524</v>
+      </c>
+      <c r="Z25" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="AA25" t="inlineStr">
+        <is>
+          <t>LastTime</t>
+        </is>
+      </c>
+      <c r="AB25" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AC25" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AD25" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AE25" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AF25" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AG25" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AH25" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AI25" t="inlineStr">
+        <is>
+          <t>SL</t>
+        </is>
+      </c>
+      <c r="AJ25" t="n">
+        <v>29112.5</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>2026-05-21</t>
+        </is>
+      </c>
+      <c r="B26" t="n">
+        <v>29193.75</v>
+      </c>
+      <c r="C26" t="n">
+        <v>29250</v>
+      </c>
+      <c r="D26" t="n">
+        <v>225</v>
+      </c>
+      <c r="E26" t="n">
+        <v>29270.18</v>
+      </c>
+      <c r="F26" t="n">
+        <v>15</v>
+      </c>
+      <c r="G26" t="n">
+        <v>849</v>
+      </c>
+      <c r="H26" t="n">
+        <v>211</v>
+      </c>
+      <c r="I26" t="inlineStr">
+        <is>
+          <t>normal speed</t>
+        </is>
+      </c>
+      <c r="J26" t="n">
+        <v>3.42</v>
+      </c>
+      <c r="K26" t="n">
+        <v>5</v>
+      </c>
+      <c r="L26" t="n">
+        <v>29238.75</v>
+      </c>
+      <c r="M26" t="n">
+        <v>29253.75</v>
+      </c>
+      <c r="N26" t="n">
+        <v>29283.75</v>
+      </c>
+      <c r="O26" t="n">
+        <v>60</v>
+      </c>
+      <c r="P26" t="n">
+        <v>120</v>
+      </c>
+      <c r="Q26" s="7" t="n">
+        <v>20</v>
+      </c>
+      <c r="R26" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="S26" t="inlineStr">
+        <is>
+          <t>BUY1</t>
+        </is>
+      </c>
+      <c r="T26" t="n">
+        <v>0</v>
+      </c>
+      <c r="U26" t="n">
+        <v>40</v>
+      </c>
+      <c r="V26" t="inlineStr">
+        <is>
+          <t>score-exporter-2026-05-25-fast-exit-half-mfe</t>
+        </is>
+      </c>
+      <c r="W26" t="inlineStr">
+        <is>
+          <t>09:52:00</t>
+        </is>
+      </c>
+      <c r="X26" t="n">
+        <v>2332</v>
+      </c>
+      <c r="Y26" t="n">
+        <v>4.3839</v>
+      </c>
+      <c r="Z26" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="AA26" t="inlineStr">
+        <is>
+          <t>LastTime</t>
+        </is>
+      </c>
+      <c r="AB26" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AC26" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AD26" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AE26" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AF26" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AG26" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="AH26" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AI26" t="inlineStr">
+        <is>
+          <t>EXIT</t>
+        </is>
+      </c>
+      <c r="AJ26" t="n">
+        <v>29258.75</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup orientation="portrait" horizontalDpi="0" verticalDpi="0"/>
 </worksheet>
 </file>
</xml_diff>